<commit_message>
Curva S actualizada 2026-09-19 13:30 Chile
</commit_message>
<xml_diff>
--- a/data/50001544 - DMC MINING SERVICES.xlsx
+++ b/data/50001544 - DMC MINING SERVICES.xlsx
@@ -2195,7 +2195,7 @@
         <v>46224.79339478009</v>
       </c>
       <c r="D10" s="5">
-        <v>46224.793407743055</v>
+        <v>46284.15352015046</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>50</v>
@@ -7941,7 +7941,7 @@
         <v>46225.55378449074</v>
       </c>
       <c r="D106" s="5">
-        <v>46225.55378673611</v>
+        <v>46284.383035844905</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>335</v>

</xml_diff>